<commit_message>
Add CRF draft Radiation Therapy
</commit_message>
<xml_diff>
--- a/curation/draft/crf/CRF_CM.xlsx
+++ b/curation/draft/crf/CRF_CM.xlsx
@@ -1,29 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\_github\cdisc-org\COSMoS\curation\draft\crf\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AD150B-4D37-4912-8208-6302F86599DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F198171-AEE0-472E-9B37-D9496A0B9A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="915" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRF_CM" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CRF_CM!$A$1:$AK$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CRF_CM!$A$1:$AK$78</definedName>
   </definedNames>
-  <calcPr calcId="0" concurrentCalc="0"/>
+  <calcPr calcId="181029" concurrentCalc="0"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1423" uniqueCount="178">
   <si>
     <t>package_date</t>
   </si>
@@ -502,12 +514,106 @@
   <si>
     <t>crf_group_id</t>
   </si>
+  <si>
+    <t>2-3</t>
+  </si>
+  <si>
+    <t>CMPRIORCANCER</t>
+  </si>
+  <si>
+    <t>CMPRIORCANCER_NORMALIZED</t>
+  </si>
+  <si>
+    <t>Free Text Anti-Cancer Therapy</t>
+  </si>
+  <si>
+    <t>Prior Anti-Cancer Therapy (Normalized)</t>
+  </si>
+  <si>
+    <t>PRIOR</t>
+  </si>
+  <si>
+    <t>CMSCAT = PRIOR</t>
+  </si>
+  <si>
+    <t>Regimen Identifier</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Concomitant Medication Name</t>
+    </r>
+  </si>
+  <si>
+    <t>No;Yes</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">ADJUVANT;METASTATIC;NEO-ADJUVANT; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri (Body)"/>
+      </rPr>
+      <t>LOCALLY ADVANCED</t>
+    </r>
+  </si>
+  <si>
+    <t>Adjuvant;Metastatic;Neo-Adjuvant;Locally Advanced</t>
+  </si>
+  <si>
+    <t>Dose per administration</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dose Unit</t>
+    </r>
+  </si>
+  <si>
+    <t>CMSTRF; CMSTRTPT;CMSTPTP</t>
+  </si>
+  <si>
+    <t>CMENRF;CMENRTPT;CMENTPT</t>
+  </si>
+  <si>
+    <t>COMPLETED PRESCRIBED REGIMEN;DISEASE PROGRESSION;TOXICITY</t>
+  </si>
+  <si>
+    <t>Completed Prescribed Regimen;Disease Progression; Toxicity</t>
+  </si>
+  <si>
+    <t>CM_ANTICANCER</t>
+  </si>
+  <si>
+    <t>Anti-Cancer Treatment specific</t>
+  </si>
+  <si>
+    <t>Concomitant Medications Yes No Indicator</t>
+  </si>
+  <si>
+    <t>Were any prior anti-cancer medications taken?</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -538,6 +644,32 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -590,7 +722,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -606,6 +738,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -908,8 +1051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:AK56"/>
+  <dimension ref="A1:AK78"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="15.42578125" customWidth="1"/>
@@ -1043,7 +1185,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:37" ht="30" hidden="1">
+    <row r="2" spans="1:37" ht="30">
       <c r="B2" t="s">
         <v>138</v>
       </c>
@@ -1099,7 +1241,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:37" ht="30" hidden="1">
+    <row r="3" spans="1:37" ht="30">
       <c r="B3" t="s">
         <v>138</v>
       </c>
@@ -1161,7 +1303,7 @@
         <v>129</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G4" t="s">
         <v>31</v>
@@ -1220,7 +1362,7 @@
         <v>129</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G5" t="s">
         <v>31</v>
@@ -1279,7 +1421,7 @@
         <v>129</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G6" t="s">
         <v>31</v>
@@ -1335,7 +1477,7 @@
         <v>129</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G7" t="s">
         <v>31</v>
@@ -1391,7 +1533,7 @@
         <v>129</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G8" t="s">
         <v>31</v>
@@ -1444,7 +1586,7 @@
         <v>129</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G9" t="s">
         <v>31</v>
@@ -1509,7 +1651,7 @@
         <v>129</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G10" t="s">
         <v>31</v>
@@ -1574,7 +1716,7 @@
         <v>129</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G11" t="s">
         <v>31</v>
@@ -1639,7 +1781,7 @@
         <v>129</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G12" t="s">
         <v>31</v>
@@ -1704,7 +1846,7 @@
         <v>129</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G13" t="s">
         <v>31</v>
@@ -1760,7 +1902,7 @@
         <v>129</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G14" t="s">
         <v>31</v>
@@ -1816,7 +1958,7 @@
         <v>129</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G15" t="s">
         <v>31</v>
@@ -1881,7 +2023,7 @@
         <v>129</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G16" t="s">
         <v>31</v>
@@ -1937,7 +2079,7 @@
         <v>129</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G17" t="s">
         <v>31</v>
@@ -1993,7 +2135,7 @@
         <v>129</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G18" t="s">
         <v>31</v>
@@ -2058,7 +2200,7 @@
         <v>129</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G19" t="s">
         <v>31</v>
@@ -2117,7 +2259,7 @@
         <v>129</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G20" t="s">
         <v>31</v>
@@ -2176,7 +2318,7 @@
         <v>129</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G21" t="s">
         <v>31</v>
@@ -2232,7 +2374,7 @@
         <v>129</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G22" t="s">
         <v>31</v>
@@ -2288,7 +2430,7 @@
         <v>129</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G23" t="s">
         <v>31</v>
@@ -2359,7 +2501,7 @@
         <v>129</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G24" t="s">
         <v>31</v>
@@ -2427,7 +2569,7 @@
         <v>129</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G25" t="s">
         <v>31</v>
@@ -2480,7 +2622,7 @@
         <v>129</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G26" t="s">
         <v>31</v>
@@ -2545,7 +2687,7 @@
         <v>129</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G27" t="s">
         <v>31</v>
@@ -2610,7 +2752,7 @@
         <v>129</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G28" t="s">
         <v>31</v>
@@ -2675,7 +2817,7 @@
         <v>129</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G29" t="s">
         <v>31</v>
@@ -2740,7 +2882,7 @@
         <v>129</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G30" t="s">
         <v>31</v>
@@ -2796,7 +2938,7 @@
         <v>129</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G31" t="s">
         <v>31</v>
@@ -2852,7 +2994,7 @@
         <v>129</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G32" t="s">
         <v>31</v>
@@ -2917,7 +3059,7 @@
         <v>129</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G33" t="s">
         <v>31</v>
@@ -2973,7 +3115,7 @@
         <v>129</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G34" t="s">
         <v>31</v>
@@ -3029,7 +3171,7 @@
         <v>129</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G35" t="s">
         <v>31</v>
@@ -3094,7 +3236,7 @@
         <v>129</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G36" t="s">
         <v>31</v>
@@ -3156,7 +3298,7 @@
         <v>129</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G37" t="s">
         <v>31</v>
@@ -3218,7 +3360,7 @@
         <v>129</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G38" t="s">
         <v>31</v>
@@ -3280,7 +3422,7 @@
         <v>129</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G39" t="s">
         <v>31</v>
@@ -3345,7 +3487,7 @@
         <v>129</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G40" t="s">
         <v>31</v>
@@ -3416,7 +3558,7 @@
         <v>129</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G41" t="s">
         <v>31</v>
@@ -3487,7 +3629,7 @@
         <v>129</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G42" t="s">
         <v>31</v>
@@ -3555,7 +3697,7 @@
         <v>129</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G43" t="s">
         <v>31</v>
@@ -3623,7 +3765,7 @@
         <v>129</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G44" t="s">
         <v>31</v>
@@ -3676,7 +3818,7 @@
         <v>129</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G45" t="s">
         <v>31</v>
@@ -3741,7 +3883,7 @@
         <v>129</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G46" t="s">
         <v>31</v>
@@ -3806,7 +3948,7 @@
         <v>129</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G47" t="s">
         <v>31</v>
@@ -3871,7 +4013,7 @@
         <v>129</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G48" t="s">
         <v>31</v>
@@ -3924,7 +4066,7 @@
         <v>129</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G49" t="s">
         <v>31</v>
@@ -3989,7 +4131,7 @@
         <v>129</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G50" t="s">
         <v>31</v>
@@ -4045,7 +4187,7 @@
         <v>129</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G51" t="s">
         <v>31</v>
@@ -4101,7 +4243,7 @@
         <v>129</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G52" t="s">
         <v>31</v>
@@ -4166,7 +4308,7 @@
         <v>129</v>
       </c>
       <c r="E53" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G53" t="s">
         <v>31</v>
@@ -4222,7 +4364,7 @@
         <v>129</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G54" t="s">
         <v>31</v>
@@ -4278,7 +4420,7 @@
         <v>129</v>
       </c>
       <c r="E55" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G55" t="s">
         <v>31</v>
@@ -4343,7 +4485,7 @@
         <v>129</v>
       </c>
       <c r="E56" s="5" t="s">
-        <v>132</v>
+        <v>156</v>
       </c>
       <c r="G56" t="s">
         <v>31</v>
@@ -4394,14 +4536,1442 @@
         <v>125</v>
       </c>
     </row>
+    <row r="57" spans="2:35">
+      <c r="B57" t="s">
+        <v>40</v>
+      </c>
+      <c r="C57" t="s">
+        <v>157</v>
+      </c>
+      <c r="D57" t="s">
+        <v>129</v>
+      </c>
+      <c r="E57" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G57" t="s">
+        <v>31</v>
+      </c>
+      <c r="H57" t="s">
+        <v>158</v>
+      </c>
+      <c r="I57" t="s">
+        <v>139</v>
+      </c>
+      <c r="J57" t="s">
+        <v>159</v>
+      </c>
+      <c r="L57" t="s">
+        <v>160</v>
+      </c>
+      <c r="M57" t="s">
+        <v>42</v>
+      </c>
+      <c r="N57" t="s">
+        <v>42</v>
+      </c>
+      <c r="O57" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q57" t="s">
+        <v>44</v>
+      </c>
+      <c r="S57">
+        <v>1</v>
+      </c>
+      <c r="T57" t="s">
+        <v>45</v>
+      </c>
+      <c r="U57" t="s">
+        <v>34</v>
+      </c>
+      <c r="V57">
+        <v>200</v>
+      </c>
+      <c r="X57" t="s">
+        <v>46</v>
+      </c>
+      <c r="AF57" t="s">
+        <v>103</v>
+      </c>
+      <c r="AH57" t="s">
+        <v>42</v>
+      </c>
+      <c r="AI57" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="58" spans="2:35">
+      <c r="B58" t="s">
+        <v>40</v>
+      </c>
+      <c r="C58" t="s">
+        <v>157</v>
+      </c>
+      <c r="D58" t="s">
+        <v>129</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G58" t="s">
+        <v>31</v>
+      </c>
+      <c r="H58" t="s">
+        <v>158</v>
+      </c>
+      <c r="I58" t="s">
+        <v>139</v>
+      </c>
+      <c r="J58" t="s">
+        <v>159</v>
+      </c>
+      <c r="L58" t="s">
+        <v>160</v>
+      </c>
+      <c r="M58" t="s">
+        <v>47</v>
+      </c>
+      <c r="N58" t="s">
+        <v>47</v>
+      </c>
+      <c r="O58" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>49</v>
+      </c>
+      <c r="S58">
+        <v>2</v>
+      </c>
+      <c r="T58" t="s">
+        <v>45</v>
+      </c>
+      <c r="U58" t="s">
+        <v>34</v>
+      </c>
+      <c r="V58">
+        <v>200</v>
+      </c>
+      <c r="X58" t="s">
+        <v>46</v>
+      </c>
+      <c r="AF58" t="s">
+        <v>161</v>
+      </c>
+      <c r="AH58" t="s">
+        <v>47</v>
+      </c>
+      <c r="AI58" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="59" spans="2:35">
+      <c r="B59" t="s">
+        <v>40</v>
+      </c>
+      <c r="C59" t="s">
+        <v>157</v>
+      </c>
+      <c r="D59" t="s">
+        <v>129</v>
+      </c>
+      <c r="E59" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G59" t="s">
+        <v>31</v>
+      </c>
+      <c r="H59" t="s">
+        <v>158</v>
+      </c>
+      <c r="I59" t="s">
+        <v>139</v>
+      </c>
+      <c r="J59" t="s">
+        <v>159</v>
+      </c>
+      <c r="L59" t="s">
+        <v>160</v>
+      </c>
+      <c r="M59" t="s">
+        <v>53</v>
+      </c>
+      <c r="N59" t="s">
+        <v>53</v>
+      </c>
+      <c r="O59" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>55</v>
+      </c>
+      <c r="S59">
+        <v>3</v>
+      </c>
+      <c r="T59" t="s">
+        <v>45</v>
+      </c>
+      <c r="U59" t="s">
+        <v>34</v>
+      </c>
+      <c r="V59">
+        <v>200</v>
+      </c>
+      <c r="X59" t="s">
+        <v>46</v>
+      </c>
+      <c r="AH59" t="s">
+        <v>53</v>
+      </c>
+      <c r="AI59" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="60" spans="2:35">
+      <c r="B60" t="s">
+        <v>40</v>
+      </c>
+      <c r="C60" t="s">
+        <v>157</v>
+      </c>
+      <c r="D60" t="s">
+        <v>129</v>
+      </c>
+      <c r="E60" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G60" t="s">
+        <v>31</v>
+      </c>
+      <c r="H60" t="s">
+        <v>158</v>
+      </c>
+      <c r="I60" t="s">
+        <v>139</v>
+      </c>
+      <c r="J60" t="s">
+        <v>159</v>
+      </c>
+      <c r="L60" t="s">
+        <v>160</v>
+      </c>
+      <c r="M60" t="s">
+        <v>105</v>
+      </c>
+      <c r="N60" t="s">
+        <v>105</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>163</v>
+      </c>
+      <c r="S60">
+        <v>4</v>
+      </c>
+      <c r="T60" t="s">
+        <v>46</v>
+      </c>
+      <c r="U60" t="s">
+        <v>34</v>
+      </c>
+      <c r="V60">
+        <v>20</v>
+      </c>
+      <c r="AC60" t="s">
+        <v>107</v>
+      </c>
+      <c r="AD60" t="s">
+        <v>107</v>
+      </c>
+      <c r="AE60" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH60" t="s">
+        <v>105</v>
+      </c>
+      <c r="AI60" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="61" spans="2:35">
+      <c r="B61" t="s">
+        <v>40</v>
+      </c>
+      <c r="C61" t="s">
+        <v>157</v>
+      </c>
+      <c r="D61" t="s">
+        <v>129</v>
+      </c>
+      <c r="E61" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G61" t="s">
+        <v>31</v>
+      </c>
+      <c r="H61" t="s">
+        <v>158</v>
+      </c>
+      <c r="I61" t="s">
+        <v>139</v>
+      </c>
+      <c r="J61" t="s">
+        <v>159</v>
+      </c>
+      <c r="L61" t="s">
+        <v>160</v>
+      </c>
+      <c r="M61" t="s">
+        <v>50</v>
+      </c>
+      <c r="N61" t="s">
+        <v>50</v>
+      </c>
+      <c r="O61" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>164</v>
+      </c>
+      <c r="S61">
+        <v>5</v>
+      </c>
+      <c r="T61" t="s">
+        <v>46</v>
+      </c>
+      <c r="U61" t="s">
+        <v>34</v>
+      </c>
+      <c r="V61">
+        <v>200</v>
+      </c>
+      <c r="AH61" t="s">
+        <v>50</v>
+      </c>
+      <c r="AI61" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="62" spans="2:35">
+      <c r="B62" t="s">
+        <v>40</v>
+      </c>
+      <c r="C62" t="s">
+        <v>157</v>
+      </c>
+      <c r="D62" t="s">
+        <v>129</v>
+      </c>
+      <c r="E62" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G62" t="s">
+        <v>31</v>
+      </c>
+      <c r="H62" t="s">
+        <v>158</v>
+      </c>
+      <c r="I62" t="s">
+        <v>139</v>
+      </c>
+      <c r="J62" t="s">
+        <v>159</v>
+      </c>
+      <c r="L62" t="s">
+        <v>160</v>
+      </c>
+      <c r="M62" t="s">
+        <v>100</v>
+      </c>
+      <c r="N62" t="s">
+        <v>100</v>
+      </c>
+      <c r="O62" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q62" t="s">
+        <v>101</v>
+      </c>
+      <c r="S62">
+        <v>6</v>
+      </c>
+      <c r="T62" t="s">
+        <v>46</v>
+      </c>
+      <c r="U62" t="s">
+        <v>34</v>
+      </c>
+      <c r="V62">
+        <v>1</v>
+      </c>
+      <c r="X62" t="s">
+        <v>46</v>
+      </c>
+      <c r="AA62" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB62" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC62" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD62" t="s">
+        <v>165</v>
+      </c>
+      <c r="AE62" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH62" t="s">
+        <v>100</v>
+      </c>
+      <c r="AI62" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="63" spans="2:35" ht="45">
+      <c r="B63" t="s">
+        <v>40</v>
+      </c>
+      <c r="C63" t="s">
+        <v>157</v>
+      </c>
+      <c r="D63" t="s">
+        <v>129</v>
+      </c>
+      <c r="E63" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G63" t="s">
+        <v>31</v>
+      </c>
+      <c r="H63" t="s">
+        <v>158</v>
+      </c>
+      <c r="I63" t="s">
+        <v>139</v>
+      </c>
+      <c r="J63" t="s">
+        <v>159</v>
+      </c>
+      <c r="L63" t="s">
+        <v>160</v>
+      </c>
+      <c r="M63" t="s">
+        <v>111</v>
+      </c>
+      <c r="N63" t="s">
+        <v>111</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>112</v>
+      </c>
+      <c r="S63">
+        <v>7</v>
+      </c>
+      <c r="T63" t="s">
+        <v>45</v>
+      </c>
+      <c r="U63" t="s">
+        <v>34</v>
+      </c>
+      <c r="V63">
+        <v>200</v>
+      </c>
+      <c r="AA63" t="s">
+        <v>113</v>
+      </c>
+      <c r="AB63" t="s">
+        <v>114</v>
+      </c>
+      <c r="AC63" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="AD63" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="AE63" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH63" t="s">
+        <v>111</v>
+      </c>
+      <c r="AI63" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="64" spans="2:35">
+      <c r="B64" t="s">
+        <v>40</v>
+      </c>
+      <c r="C64" t="s">
+        <v>157</v>
+      </c>
+      <c r="D64" t="s">
+        <v>129</v>
+      </c>
+      <c r="E64" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G64" t="s">
+        <v>31</v>
+      </c>
+      <c r="H64" t="s">
+        <v>158</v>
+      </c>
+      <c r="I64" t="s">
+        <v>139</v>
+      </c>
+      <c r="J64" t="s">
+        <v>159</v>
+      </c>
+      <c r="L64" t="s">
+        <v>160</v>
+      </c>
+      <c r="M64" t="s">
+        <v>117</v>
+      </c>
+      <c r="N64" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q64" t="s">
+        <v>118</v>
+      </c>
+      <c r="S64">
+        <v>8</v>
+      </c>
+      <c r="T64" t="s">
+        <v>45</v>
+      </c>
+      <c r="U64" t="s">
+        <v>34</v>
+      </c>
+      <c r="V64">
+        <v>200</v>
+      </c>
+      <c r="AA64" t="s">
+        <v>119</v>
+      </c>
+      <c r="AB64" t="s">
+        <v>120</v>
+      </c>
+      <c r="AC64" t="s">
+        <v>121</v>
+      </c>
+      <c r="AD64" t="s">
+        <v>122</v>
+      </c>
+      <c r="AE64" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH64" t="s">
+        <v>117</v>
+      </c>
+      <c r="AI64" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="65" spans="2:35">
+      <c r="B65" t="s">
+        <v>40</v>
+      </c>
+      <c r="C65" t="s">
+        <v>157</v>
+      </c>
+      <c r="D65" t="s">
+        <v>129</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G65" t="s">
+        <v>31</v>
+      </c>
+      <c r="H65" t="s">
+        <v>158</v>
+      </c>
+      <c r="I65" t="s">
+        <v>139</v>
+      </c>
+      <c r="J65" t="s">
+        <v>159</v>
+      </c>
+      <c r="L65" t="s">
+        <v>160</v>
+      </c>
+      <c r="M65" t="s">
+        <v>56</v>
+      </c>
+      <c r="N65" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q65" t="s">
+        <v>168</v>
+      </c>
+      <c r="S65">
+        <v>9</v>
+      </c>
+      <c r="T65" t="s">
+        <v>46</v>
+      </c>
+      <c r="U65" t="s">
+        <v>34</v>
+      </c>
+      <c r="V65">
+        <v>100</v>
+      </c>
+      <c r="AH65" t="s">
+        <v>58</v>
+      </c>
+      <c r="AI65" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="66" spans="2:35">
+      <c r="B66" t="s">
+        <v>40</v>
+      </c>
+      <c r="C66" t="s">
+        <v>157</v>
+      </c>
+      <c r="D66" t="s">
+        <v>129</v>
+      </c>
+      <c r="E66" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G66" t="s">
+        <v>31</v>
+      </c>
+      <c r="H66" t="s">
+        <v>158</v>
+      </c>
+      <c r="I66" t="s">
+        <v>139</v>
+      </c>
+      <c r="J66" t="s">
+        <v>159</v>
+      </c>
+      <c r="L66" t="s">
+        <v>160</v>
+      </c>
+      <c r="M66" t="s">
+        <v>59</v>
+      </c>
+      <c r="N66" t="s">
+        <v>59</v>
+      </c>
+      <c r="O66" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q66" t="s">
+        <v>169</v>
+      </c>
+      <c r="S66">
+        <v>10</v>
+      </c>
+      <c r="T66" t="s">
+        <v>46</v>
+      </c>
+      <c r="U66" t="s">
+        <v>34</v>
+      </c>
+      <c r="V66">
+        <v>40</v>
+      </c>
+      <c r="AA66" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB66" t="s">
+        <v>63</v>
+      </c>
+      <c r="AC66" s="8"/>
+      <c r="AD66" s="8"/>
+      <c r="AE66" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH66" t="s">
+        <v>59</v>
+      </c>
+      <c r="AI66" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="67" spans="2:35">
+      <c r="B67" t="s">
+        <v>40</v>
+      </c>
+      <c r="C67" t="s">
+        <v>157</v>
+      </c>
+      <c r="D67" t="s">
+        <v>129</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G67" t="s">
+        <v>31</v>
+      </c>
+      <c r="H67" t="s">
+        <v>158</v>
+      </c>
+      <c r="I67" t="s">
+        <v>139</v>
+      </c>
+      <c r="J67" t="s">
+        <v>159</v>
+      </c>
+      <c r="L67" t="s">
+        <v>160</v>
+      </c>
+      <c r="M67" t="s">
+        <v>64</v>
+      </c>
+      <c r="N67" t="s">
+        <v>64</v>
+      </c>
+      <c r="O67" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q67" t="s">
+        <v>66</v>
+      </c>
+      <c r="S67">
+        <v>11</v>
+      </c>
+      <c r="T67" t="s">
+        <v>45</v>
+      </c>
+      <c r="U67" t="s">
+        <v>34</v>
+      </c>
+      <c r="V67">
+        <v>40</v>
+      </c>
+      <c r="AA67" t="s">
+        <v>67</v>
+      </c>
+      <c r="AB67" t="s">
+        <v>68</v>
+      </c>
+      <c r="AC67" s="8"/>
+      <c r="AD67" s="8"/>
+      <c r="AE67" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH67" t="s">
+        <v>64</v>
+      </c>
+      <c r="AI67" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="68" spans="2:35">
+      <c r="B68" t="s">
+        <v>40</v>
+      </c>
+      <c r="C68" t="s">
+        <v>157</v>
+      </c>
+      <c r="D68" t="s">
+        <v>129</v>
+      </c>
+      <c r="E68" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G68" t="s">
+        <v>31</v>
+      </c>
+      <c r="H68" t="s">
+        <v>158</v>
+      </c>
+      <c r="I68" t="s">
+        <v>139</v>
+      </c>
+      <c r="J68" t="s">
+        <v>159</v>
+      </c>
+      <c r="L68" t="s">
+        <v>160</v>
+      </c>
+      <c r="M68" t="s">
+        <v>69</v>
+      </c>
+      <c r="N68" t="s">
+        <v>69</v>
+      </c>
+      <c r="O68" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>71</v>
+      </c>
+      <c r="S68">
+        <v>12</v>
+      </c>
+      <c r="T68" t="s">
+        <v>45</v>
+      </c>
+      <c r="U68" t="s">
+        <v>34</v>
+      </c>
+      <c r="V68">
+        <v>40</v>
+      </c>
+      <c r="AA68" t="s">
+        <v>72</v>
+      </c>
+      <c r="AB68" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC68" s="8"/>
+      <c r="AD68" s="8"/>
+      <c r="AE68" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH68" t="s">
+        <v>69</v>
+      </c>
+      <c r="AI68" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="69" spans="2:35" ht="15.75">
+      <c r="B69" t="s">
+        <v>40</v>
+      </c>
+      <c r="C69" t="s">
+        <v>157</v>
+      </c>
+      <c r="D69" t="s">
+        <v>129</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G69" t="s">
+        <v>31</v>
+      </c>
+      <c r="H69" t="s">
+        <v>158</v>
+      </c>
+      <c r="I69" t="s">
+        <v>139</v>
+      </c>
+      <c r="J69" t="s">
+        <v>159</v>
+      </c>
+      <c r="L69" t="s">
+        <v>160</v>
+      </c>
+      <c r="M69" t="s">
+        <v>123</v>
+      </c>
+      <c r="N69" t="s">
+        <v>123</v>
+      </c>
+      <c r="Q69" t="s">
+        <v>124</v>
+      </c>
+      <c r="S69">
+        <v>13</v>
+      </c>
+      <c r="T69" t="s">
+        <v>45</v>
+      </c>
+      <c r="U69" t="s">
+        <v>34</v>
+      </c>
+      <c r="V69">
+        <v>200</v>
+      </c>
+      <c r="AC69" s="9"/>
+      <c r="AD69" s="9"/>
+      <c r="AE69" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH69" t="s">
+        <v>123</v>
+      </c>
+      <c r="AI69" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="70" spans="2:35" ht="15.75">
+      <c r="B70" t="s">
+        <v>40</v>
+      </c>
+      <c r="C70" t="s">
+        <v>157</v>
+      </c>
+      <c r="D70" t="s">
+        <v>129</v>
+      </c>
+      <c r="E70" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G70" t="s">
+        <v>31</v>
+      </c>
+      <c r="H70" t="s">
+        <v>158</v>
+      </c>
+      <c r="I70" t="s">
+        <v>139</v>
+      </c>
+      <c r="J70" t="s">
+        <v>159</v>
+      </c>
+      <c r="L70" t="s">
+        <v>160</v>
+      </c>
+      <c r="M70" t="s">
+        <v>74</v>
+      </c>
+      <c r="N70" t="s">
+        <v>74</v>
+      </c>
+      <c r="O70" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q70" t="s">
+        <v>76</v>
+      </c>
+      <c r="S70">
+        <v>14</v>
+      </c>
+      <c r="T70" t="s">
+        <v>45</v>
+      </c>
+      <c r="U70" t="s">
+        <v>34</v>
+      </c>
+      <c r="V70">
+        <v>200</v>
+      </c>
+      <c r="AA70" t="s">
+        <v>77</v>
+      </c>
+      <c r="AB70" t="s">
+        <v>78</v>
+      </c>
+      <c r="AC70" s="10"/>
+      <c r="AD70" s="8"/>
+      <c r="AE70" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH70" t="s">
+        <v>74</v>
+      </c>
+      <c r="AI70" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="71" spans="2:35">
+      <c r="B71" t="s">
+        <v>40</v>
+      </c>
+      <c r="C71" t="s">
+        <v>157</v>
+      </c>
+      <c r="D71" t="s">
+        <v>129</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G71" t="s">
+        <v>31</v>
+      </c>
+      <c r="H71" t="s">
+        <v>158</v>
+      </c>
+      <c r="I71" t="s">
+        <v>139</v>
+      </c>
+      <c r="J71" t="s">
+        <v>159</v>
+      </c>
+      <c r="L71" t="s">
+        <v>160</v>
+      </c>
+      <c r="M71" t="s">
+        <v>79</v>
+      </c>
+      <c r="N71" t="s">
+        <v>80</v>
+      </c>
+      <c r="O71" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q71" t="s">
+        <v>82</v>
+      </c>
+      <c r="S71">
+        <v>15</v>
+      </c>
+      <c r="T71" t="s">
+        <v>46</v>
+      </c>
+      <c r="U71" t="s">
+        <v>83</v>
+      </c>
+      <c r="V71">
+        <v>10</v>
+      </c>
+      <c r="AH71" t="s">
+        <v>80</v>
+      </c>
+      <c r="AI71" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="72" spans="2:35">
+      <c r="B72" t="s">
+        <v>40</v>
+      </c>
+      <c r="C72" t="s">
+        <v>157</v>
+      </c>
+      <c r="D72" t="s">
+        <v>129</v>
+      </c>
+      <c r="E72" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G72" t="s">
+        <v>31</v>
+      </c>
+      <c r="H72" t="s">
+        <v>158</v>
+      </c>
+      <c r="I72" t="s">
+        <v>139</v>
+      </c>
+      <c r="J72" t="s">
+        <v>159</v>
+      </c>
+      <c r="L72" t="s">
+        <v>160</v>
+      </c>
+      <c r="M72" t="s">
+        <v>84</v>
+      </c>
+      <c r="N72" t="s">
+        <v>80</v>
+      </c>
+      <c r="O72" t="s">
+        <v>81</v>
+      </c>
+      <c r="Q72" t="s">
+        <v>85</v>
+      </c>
+      <c r="S72">
+        <v>16</v>
+      </c>
+      <c r="T72" t="s">
+        <v>45</v>
+      </c>
+      <c r="U72" t="s">
+        <v>86</v>
+      </c>
+      <c r="V72">
+        <v>5</v>
+      </c>
+      <c r="AH72" t="s">
+        <v>80</v>
+      </c>
+      <c r="AI72" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="73" spans="2:35">
+      <c r="B73" t="s">
+        <v>40</v>
+      </c>
+      <c r="C73" t="s">
+        <v>157</v>
+      </c>
+      <c r="D73" t="s">
+        <v>129</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G73" t="s">
+        <v>31</v>
+      </c>
+      <c r="H73" t="s">
+        <v>158</v>
+      </c>
+      <c r="I73" t="s">
+        <v>139</v>
+      </c>
+      <c r="J73" t="s">
+        <v>159</v>
+      </c>
+      <c r="L73" t="s">
+        <v>160</v>
+      </c>
+      <c r="M73" t="s">
+        <v>87</v>
+      </c>
+      <c r="N73" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q73" t="s">
+        <v>88</v>
+      </c>
+      <c r="S73">
+        <v>17</v>
+      </c>
+      <c r="T73" t="s">
+        <v>45</v>
+      </c>
+      <c r="U73" t="s">
+        <v>34</v>
+      </c>
+      <c r="V73">
+        <v>1</v>
+      </c>
+      <c r="X73" t="s">
+        <v>46</v>
+      </c>
+      <c r="AA73" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB73" t="s">
+        <v>36</v>
+      </c>
+      <c r="AF73" t="s">
+        <v>46</v>
+      </c>
+      <c r="AH73" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="AI73" s="11" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="74" spans="2:35">
+      <c r="B74" t="s">
+        <v>40</v>
+      </c>
+      <c r="C74" t="s">
+        <v>157</v>
+      </c>
+      <c r="D74" t="s">
+        <v>129</v>
+      </c>
+      <c r="E74" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G74" t="s">
+        <v>31</v>
+      </c>
+      <c r="H74" t="s">
+        <v>158</v>
+      </c>
+      <c r="I74" t="s">
+        <v>139</v>
+      </c>
+      <c r="J74" t="s">
+        <v>159</v>
+      </c>
+      <c r="L74" t="s">
+        <v>160</v>
+      </c>
+      <c r="M74" t="s">
+        <v>89</v>
+      </c>
+      <c r="N74" t="s">
+        <v>90</v>
+      </c>
+      <c r="O74" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q74" t="s">
+        <v>92</v>
+      </c>
+      <c r="S74">
+        <v>18</v>
+      </c>
+      <c r="T74" t="s">
+        <v>45</v>
+      </c>
+      <c r="U74" t="s">
+        <v>83</v>
+      </c>
+      <c r="V74">
+        <v>10</v>
+      </c>
+      <c r="AH74" t="s">
+        <v>90</v>
+      </c>
+      <c r="AI74" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="75" spans="2:35">
+      <c r="B75" t="s">
+        <v>40</v>
+      </c>
+      <c r="C75" t="s">
+        <v>157</v>
+      </c>
+      <c r="D75" t="s">
+        <v>129</v>
+      </c>
+      <c r="E75" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G75" t="s">
+        <v>31</v>
+      </c>
+      <c r="H75" t="s">
+        <v>158</v>
+      </c>
+      <c r="I75" t="s">
+        <v>139</v>
+      </c>
+      <c r="J75" t="s">
+        <v>159</v>
+      </c>
+      <c r="L75" t="s">
+        <v>160</v>
+      </c>
+      <c r="M75" t="s">
+        <v>93</v>
+      </c>
+      <c r="N75" t="s">
+        <v>90</v>
+      </c>
+      <c r="O75" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q75" t="s">
+        <v>94</v>
+      </c>
+      <c r="S75">
+        <v>19</v>
+      </c>
+      <c r="T75" t="s">
+        <v>45</v>
+      </c>
+      <c r="U75" t="s">
+        <v>86</v>
+      </c>
+      <c r="V75">
+        <v>5</v>
+      </c>
+      <c r="AH75" t="s">
+        <v>90</v>
+      </c>
+      <c r="AI75" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="76" spans="2:35">
+      <c r="B76" t="s">
+        <v>40</v>
+      </c>
+      <c r="C76" t="s">
+        <v>157</v>
+      </c>
+      <c r="D76" t="s">
+        <v>129</v>
+      </c>
+      <c r="E76" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G76" t="s">
+        <v>31</v>
+      </c>
+      <c r="H76" t="s">
+        <v>158</v>
+      </c>
+      <c r="I76" t="s">
+        <v>139</v>
+      </c>
+      <c r="J76" t="s">
+        <v>159</v>
+      </c>
+      <c r="L76" t="s">
+        <v>160</v>
+      </c>
+      <c r="M76" t="s">
+        <v>95</v>
+      </c>
+      <c r="N76" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q76" t="s">
+        <v>96</v>
+      </c>
+      <c r="S76">
+        <v>20</v>
+      </c>
+      <c r="T76" t="s">
+        <v>45</v>
+      </c>
+      <c r="U76" t="s">
+        <v>34</v>
+      </c>
+      <c r="V76">
+        <v>1</v>
+      </c>
+      <c r="AA76" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB76" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC76" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD76" t="s">
+        <v>165</v>
+      </c>
+      <c r="AE76" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH76" t="s">
+        <v>147</v>
+      </c>
+      <c r="AI76" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="77" spans="2:35" ht="45">
+      <c r="B77" t="s">
+        <v>40</v>
+      </c>
+      <c r="C77" t="s">
+        <v>157</v>
+      </c>
+      <c r="D77" t="s">
+        <v>129</v>
+      </c>
+      <c r="E77" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G77" t="s">
+        <v>31</v>
+      </c>
+      <c r="H77" t="s">
+        <v>158</v>
+      </c>
+      <c r="I77" t="s">
+        <v>139</v>
+      </c>
+      <c r="J77" t="s">
+        <v>159</v>
+      </c>
+      <c r="L77" t="s">
+        <v>160</v>
+      </c>
+      <c r="M77" t="s">
+        <v>125</v>
+      </c>
+      <c r="N77" t="s">
+        <v>125</v>
+      </c>
+      <c r="Q77" t="s">
+        <v>126</v>
+      </c>
+      <c r="S77">
+        <v>21</v>
+      </c>
+      <c r="T77" t="s">
+        <v>45</v>
+      </c>
+      <c r="U77" t="s">
+        <v>34</v>
+      </c>
+      <c r="V77">
+        <v>200</v>
+      </c>
+      <c r="AC77" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="AD77" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="AE77" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH77" t="s">
+        <v>125</v>
+      </c>
+      <c r="AI77" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="78" spans="2:35" ht="45">
+      <c r="B78" t="s">
+        <v>138</v>
+      </c>
+      <c r="D78" t="s">
+        <v>129</v>
+      </c>
+      <c r="E78" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="G78" t="s">
+        <v>31</v>
+      </c>
+      <c r="H78" t="s">
+        <v>174</v>
+      </c>
+      <c r="J78" t="s">
+        <v>175</v>
+      </c>
+      <c r="L78" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="M78" t="s">
+        <v>32</v>
+      </c>
+      <c r="N78" t="s">
+        <v>32</v>
+      </c>
+      <c r="P78" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="S78">
+        <v>1</v>
+      </c>
+      <c r="T78" t="s">
+        <v>46</v>
+      </c>
+      <c r="U78" t="s">
+        <v>34</v>
+      </c>
+      <c r="V78">
+        <v>1</v>
+      </c>
+      <c r="AA78" t="s">
+        <v>35</v>
+      </c>
+      <c r="AB78" t="s">
+        <v>36</v>
+      </c>
+      <c r="AC78" t="s">
+        <v>37</v>
+      </c>
+      <c r="AD78" t="s">
+        <v>165</v>
+      </c>
+      <c r="AE78" t="s">
+        <v>38</v>
+      </c>
+      <c r="AI78" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AK56" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="C53630"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:AK78" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>